<commit_message>
content: expand leadership approach to 24 questions
</commit_message>
<xml_diff>
--- a/content/assessment-packages/leadership-approach/sonartra_reader_first_import_schema_LEADERSHIP_APPROACH_TEST.xlsx
+++ b/content/assessment-packages/leadership-approach/sonartra_reader_first_import_schema_LEADERSHIP_APPROACH_TEST.xlsx
@@ -19176,7 +19176,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:F25"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -19209,7 +19209,7 @@
         <v>1</v>
       </c>
       <c r="D2" t="str">
-        <v>When a leadership situation becomes unclear, what do you tend to clarify first?</v>
+        <v>When leading a team, what do you focus on most?</v>
       </c>
       <c r="E2" t="str">
         <v>active</v>
@@ -19229,7 +19229,7 @@
         <v>2</v>
       </c>
       <c r="D3" t="str">
-        <v>When a team needs momentum, what do you usually bring into the room first?</v>
+        <v>How do you define success for your team?</v>
       </c>
       <c r="E3" t="str">
         <v>active</v>
@@ -19249,7 +19249,7 @@
         <v>3</v>
       </c>
       <c r="D4" t="str">
-        <v>When pressure rises, what do you most want to protect?</v>
+        <v>When things are not working well, what is your instinct?</v>
       </c>
       <c r="E4" t="str">
         <v>active</v>
@@ -19269,7 +19269,7 @@
         <v>4</v>
       </c>
       <c r="D5" t="str">
-        <v>When a decision has to move forward, what do you naturally check first?</v>
+        <v>In meetings, how do you tend to lead?</v>
       </c>
       <c r="E5" t="str">
         <v>active</v>
@@ -19289,7 +19289,7 @@
         <v>5</v>
       </c>
       <c r="D6" t="str">
-        <v>When others are looking for direction, what do you usually make visible first?</v>
+        <v>When setting expectations, what matters most?</v>
       </c>
       <c r="E6" t="str">
         <v>active</v>
@@ -19309,7 +19309,7 @@
         <v>6</v>
       </c>
       <c r="D7" t="str">
-        <v>When work starts to drift, what is your first corrective move?</v>
+        <v>What do you tend to emphasise with your team?</v>
       </c>
       <c r="E7" t="str">
         <v>active</v>
@@ -19329,7 +19329,7 @@
         <v>7</v>
       </c>
       <c r="D8" t="str">
-        <v>When change is needed, what do you tend to emphasise first?</v>
+        <v>When making decisions, what do you prioritise?</v>
       </c>
       <c r="E8" t="str">
         <v>active</v>
@@ -19349,7 +19349,7 @@
         <v>8</v>
       </c>
       <c r="D9" t="str">
-        <v>When people disagree, what do you usually try to restore first?</v>
+        <v>How do you help people stay accountable?</v>
       </c>
       <c r="E9" t="str">
         <v>active</v>
@@ -19369,7 +19369,7 @@
         <v>9</v>
       </c>
       <c r="D10" t="str">
-        <v>When a plan is forming, what do you trust most as the starting point?</v>
+        <v>What do others rely on you for most as a leader?</v>
       </c>
       <c r="E10" t="str">
         <v>active</v>
@@ -19389,7 +19389,7 @@
         <v>10</v>
       </c>
       <c r="D11" t="str">
-        <v>When progress stalls, what kind of leadership action feels most useful?</v>
+        <v>How would others describe your leadership style?</v>
       </c>
       <c r="E11" t="str">
         <v>active</v>
@@ -19409,7 +19409,7 @@
         <v>11</v>
       </c>
       <c r="D12" t="str">
-        <v>When a group needs confidence, what do you usually provide first?</v>
+        <v>Under pressure, how do you lead?</v>
       </c>
       <c r="E12" t="str">
         <v>active</v>
@@ -19429,7 +19429,7 @@
         <v>12</v>
       </c>
       <c r="D13" t="str">
-        <v>When the next step is uncertain, what do you naturally reach for?</v>
+        <v>When priorities compete, what matters most to you?</v>
       </c>
       <c r="E13" t="str">
         <v>active</v>
@@ -19449,7 +19449,7 @@
         <v>13</v>
       </c>
       <c r="D14" t="str">
-        <v>When a project gets complex, what do you notice earliest?</v>
+        <v>What frustrates you most in a team?</v>
       </c>
       <c r="E14" t="str">
         <v>active</v>
@@ -19469,7 +19469,7 @@
         <v>14</v>
       </c>
       <c r="D15" t="str">
-        <v>When responsibility is shared, what do you most want to make explicit?</v>
+        <v>What gives you confidence in a team?</v>
       </c>
       <c r="E15" t="str">
         <v>active</v>
@@ -19489,7 +19489,7 @@
         <v>15</v>
       </c>
       <c r="D16" t="str">
-        <v>When standards are at risk, what do you tend to do first?</v>
+        <v>What do you try hardest to protect as a leader?</v>
       </c>
       <c r="E16" t="str">
         <v>active</v>
@@ -19509,7 +19509,7 @@
         <v>16</v>
       </c>
       <c r="D17" t="str">
-        <v>When the work needs commitment, what do you usually strengthen first?</v>
+        <v>When your plan is challenged, what is your instinct?</v>
       </c>
       <c r="E17" t="str">
         <v>active</v>
@@ -19518,16 +19518,176 @@
         <v>leadership_approach::q16</v>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>leadership_approach</v>
+      </c>
+      <c r="B18" t="str">
+        <v>leadership_approach_q17</v>
+      </c>
+      <c r="C18">
+        <v>17</v>
+      </c>
+      <c r="D18" t="str">
+        <v>When time is tight, what do you adjust first?</v>
+      </c>
+      <c r="E18" t="str">
+        <v>active</v>
+      </c>
+      <c r="F18" t="str">
+        <v>leadership_approach::q17</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>leadership_approach</v>
+      </c>
+      <c r="B19" t="str">
+        <v>leadership_approach_q18</v>
+      </c>
+      <c r="C19">
+        <v>18</v>
+      </c>
+      <c r="D19" t="str">
+        <v>When work stalls, what do you look at first?</v>
+      </c>
+      <c r="E19" t="str">
+        <v>active</v>
+      </c>
+      <c r="F19" t="str">
+        <v>leadership_approach::q18</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>leadership_approach</v>
+      </c>
+      <c r="B20" t="str">
+        <v>leadership_approach_q19</v>
+      </c>
+      <c r="C20">
+        <v>19</v>
+      </c>
+      <c r="D20" t="str">
+        <v>When people disagree, how do you respond?</v>
+      </c>
+      <c r="E20" t="str">
+        <v>active</v>
+      </c>
+      <c r="F20" t="str">
+        <v>leadership_approach::q19</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>leadership_approach</v>
+      </c>
+      <c r="B21" t="str">
+        <v>leadership_approach_q20</v>
+      </c>
+      <c r="C21">
+        <v>20</v>
+      </c>
+      <c r="D21" t="str">
+        <v>What tends to concern you most in a team?</v>
+      </c>
+      <c r="E21" t="str">
+        <v>active</v>
+      </c>
+      <c r="F21" t="str">
+        <v>leadership_approach::q20</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>leadership_approach</v>
+      </c>
+      <c r="B22" t="str">
+        <v>leadership_approach_q21</v>
+      </c>
+      <c r="C22">
+        <v>21</v>
+      </c>
+      <c r="D22" t="str">
+        <v>When progress slows, what do you focus on next?</v>
+      </c>
+      <c r="E22" t="str">
+        <v>active</v>
+      </c>
+      <c r="F22" t="str">
+        <v>leadership_approach::q21</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>leadership_approach</v>
+      </c>
+      <c r="B23" t="str">
+        <v>leadership_approach_q22</v>
+      </c>
+      <c r="C23">
+        <v>22</v>
+      </c>
+      <c r="D23" t="str">
+        <v>When starting new work, what do you establish first?</v>
+      </c>
+      <c r="E23" t="str">
+        <v>active</v>
+      </c>
+      <c r="F23" t="str">
+        <v>leadership_approach::q22</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>leadership_approach</v>
+      </c>
+      <c r="B24" t="str">
+        <v>leadership_approach_q23</v>
+      </c>
+      <c r="C24">
+        <v>23</v>
+      </c>
+      <c r="D24" t="str">
+        <v>When something goes wrong, what do you focus on first?</v>
+      </c>
+      <c r="E24" t="str">
+        <v>active</v>
+      </c>
+      <c r="F24" t="str">
+        <v>leadership_approach::q23</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>leadership_approach</v>
+      </c>
+      <c r="B25" t="str">
+        <v>leadership_approach_q24</v>
+      </c>
+      <c r="C25">
+        <v>24</v>
+      </c>
+      <c r="D25" t="str">
+        <v>When work is going well, what do you reinforce?</v>
+      </c>
+      <c r="E25" t="str">
+        <v>active</v>
+      </c>
+      <c r="F25" t="str">
+        <v>leadership_approach::q24</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F17"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F25"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H65"/>
+  <dimension ref="A1:H97"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -19569,7 +19729,7 @@
         <v>A</v>
       </c>
       <c r="E2" t="str">
-        <v>The outcome, owner, decision, and next visible move.</v>
+        <v>Clarify what needs to be delivered</v>
       </c>
       <c r="F2" t="str">
         <v>true</v>
@@ -19595,7 +19755,7 @@
         <v>B</v>
       </c>
       <c r="E3" t="str">
-        <v>The structure, sequence, standard, and reliable way of working.</v>
+        <v>Clarify where the work is heading</v>
       </c>
       <c r="F3" t="str">
         <v>true</v>
@@ -19621,7 +19781,7 @@
         <v>C</v>
       </c>
       <c r="E4" t="str">
-        <v>The future direction, wider meaning, and frame for the choice.</v>
+        <v>Set out how the work should run</v>
       </c>
       <c r="F4" t="str">
         <v>true</v>
@@ -19647,7 +19807,7 @@
         <v>D</v>
       </c>
       <c r="E5" t="str">
-        <v>The trust, communication, involvement, and effect on people.</v>
+        <v>Check what people need to contribute</v>
       </c>
       <c r="F5" t="str">
         <v>true</v>
@@ -19673,7 +19833,7 @@
         <v>A</v>
       </c>
       <c r="E6" t="str">
-        <v>The outcome, owner, decision, and next visible move.</v>
+        <v>Work runs in a consistent way</v>
       </c>
       <c r="F6" t="str">
         <v>true</v>
@@ -19699,7 +19859,7 @@
         <v>B</v>
       </c>
       <c r="E7" t="str">
-        <v>The structure, sequence, standard, and reliable way of working.</v>
+        <v>Effort leads to clear outcomes</v>
       </c>
       <c r="F7" t="str">
         <v>true</v>
@@ -19725,7 +19885,7 @@
         <v>C</v>
       </c>
       <c r="E8" t="str">
-        <v>The future direction, wider meaning, and frame for the choice.</v>
+        <v>People grow and stay engaged</v>
       </c>
       <c r="F8" t="str">
         <v>true</v>
@@ -19751,7 +19911,7 @@
         <v>D</v>
       </c>
       <c r="E9" t="str">
-        <v>The trust, communication, involvement, and effect on people.</v>
+        <v>Work moves in the right direction</v>
       </c>
       <c r="F9" t="str">
         <v>true</v>
@@ -19777,7 +19937,7 @@
         <v>A</v>
       </c>
       <c r="E10" t="str">
-        <v>The outcome, owner, decision, and next visible move.</v>
+        <v>Check what people need first</v>
       </c>
       <c r="F10" t="str">
         <v>true</v>
@@ -19803,7 +19963,7 @@
         <v>B</v>
       </c>
       <c r="E11" t="str">
-        <v>The structure, sequence, standard, and reliable way of working.</v>
+        <v>Look at how the work is running</v>
       </c>
       <c r="F11" t="str">
         <v>true</v>
@@ -19829,7 +19989,7 @@
         <v>C</v>
       </c>
       <c r="E12" t="str">
-        <v>The future direction, wider meaning, and frame for the choice.</v>
+        <v>Focus on what needs to happen next</v>
       </c>
       <c r="F12" t="str">
         <v>true</v>
@@ -19855,7 +20015,7 @@
         <v>D</v>
       </c>
       <c r="E13" t="str">
-        <v>The trust, communication, involvement, and effect on people.</v>
+        <v>Step back and check the direction</v>
       </c>
       <c r="F13" t="str">
         <v>true</v>
@@ -19881,7 +20041,7 @@
         <v>A</v>
       </c>
       <c r="E14" t="str">
-        <v>The outcome, owner, decision, and next visible move.</v>
+        <v>Keep the conversation clearly organised</v>
       </c>
       <c r="F14" t="str">
         <v>true</v>
@@ -19907,7 +20067,7 @@
         <v>B</v>
       </c>
       <c r="E15" t="str">
-        <v>The structure, sequence, standard, and reliable way of working.</v>
+        <v>Make space for people to be heard</v>
       </c>
       <c r="F15" t="str">
         <v>true</v>
@@ -19933,7 +20093,7 @@
         <v>C</v>
       </c>
       <c r="E16" t="str">
-        <v>The future direction, wider meaning, and frame for the choice.</v>
+        <v>Keep focus on decisions and next steps</v>
       </c>
       <c r="F16" t="str">
         <v>true</v>
@@ -19959,7 +20119,7 @@
         <v>D</v>
       </c>
       <c r="E17" t="str">
-        <v>The trust, communication, involvement, and effect on people.</v>
+        <v>Connect the discussion to the wider direction</v>
       </c>
       <c r="F17" t="str">
         <v>true</v>
@@ -19985,7 +20145,7 @@
         <v>A</v>
       </c>
       <c r="E18" t="str">
-        <v>The outcome, owner, decision, and next visible move.</v>
+        <v>Understand what people need to contribute</v>
       </c>
       <c r="F18" t="str">
         <v>true</v>
@@ -20011,7 +20171,7 @@
         <v>B</v>
       </c>
       <c r="E19" t="str">
-        <v>The structure, sequence, standard, and reliable way of working.</v>
+        <v>Make the expected outcome clear</v>
       </c>
       <c r="F19" t="str">
         <v>true</v>
@@ -20037,7 +20197,7 @@
         <v>C</v>
       </c>
       <c r="E20" t="str">
-        <v>The future direction, wider meaning, and frame for the choice.</v>
+        <v>Make roles and ways of working clear</v>
       </c>
       <c r="F20" t="str">
         <v>true</v>
@@ -20063,7 +20223,7 @@
         <v>D</v>
       </c>
       <c r="E21" t="str">
-        <v>The trust, communication, involvement, and effect on people.</v>
+        <v>Make the direction and purpose clear</v>
       </c>
       <c r="F21" t="str">
         <v>true</v>
@@ -20089,7 +20249,7 @@
         <v>A</v>
       </c>
       <c r="E22" t="str">
-        <v>The outcome, owner, decision, and next visible move.</v>
+        <v>Where the work is heading</v>
       </c>
       <c r="F22" t="str">
         <v>true</v>
@@ -20115,7 +20275,7 @@
         <v>B</v>
       </c>
       <c r="E23" t="str">
-        <v>The structure, sequence, standard, and reliable way of working.</v>
+        <v>How the work should run</v>
       </c>
       <c r="F23" t="str">
         <v>true</v>
@@ -20141,7 +20301,7 @@
         <v>C</v>
       </c>
       <c r="E24" t="str">
-        <v>The future direction, wider meaning, and frame for the choice.</v>
+        <v>What needs to be delivered</v>
       </c>
       <c r="F24" t="str">
         <v>true</v>
@@ -20167,7 +20327,7 @@
         <v>D</v>
       </c>
       <c r="E25" t="str">
-        <v>The trust, communication, involvement, and effect on people.</v>
+        <v>What people need to contribute</v>
       </c>
       <c r="F25" t="str">
         <v>true</v>
@@ -20193,7 +20353,7 @@
         <v>A</v>
       </c>
       <c r="E26" t="str">
-        <v>The outcome, owner, decision, and next visible move.</v>
+        <v>What people need to move forward</v>
       </c>
       <c r="F26" t="str">
         <v>true</v>
@@ -20219,7 +20379,7 @@
         <v>B</v>
       </c>
       <c r="E27" t="str">
-        <v>The structure, sequence, standard, and reliable way of working.</v>
+        <v>What will make the approach reliable</v>
       </c>
       <c r="F27" t="str">
         <v>true</v>
@@ -20245,7 +20405,7 @@
         <v>C</v>
       </c>
       <c r="E28" t="str">
-        <v>The future direction, wider meaning, and frame for the choice.</v>
+        <v>What will produce the clearest outcome</v>
       </c>
       <c r="F28" t="str">
         <v>true</v>
@@ -20271,7 +20431,7 @@
         <v>D</v>
       </c>
       <c r="E29" t="str">
-        <v>The trust, communication, involvement, and effect on people.</v>
+        <v>What fits the wider direction</v>
       </c>
       <c r="F29" t="str">
         <v>true</v>
@@ -20297,7 +20457,7 @@
         <v>A</v>
       </c>
       <c r="E30" t="str">
-        <v>The outcome, owner, decision, and next visible move.</v>
+        <v>Set clear ways of working</v>
       </c>
       <c r="F30" t="str">
         <v>true</v>
@@ -20323,7 +20483,7 @@
         <v>B</v>
       </c>
       <c r="E31" t="str">
-        <v>The structure, sequence, standard, and reliable way of working.</v>
+        <v>Set a clear standard for the work</v>
       </c>
       <c r="F31" t="str">
         <v>true</v>
@@ -20349,7 +20509,7 @@
         <v>C</v>
       </c>
       <c r="E32" t="str">
-        <v>The future direction, wider meaning, and frame for the choice.</v>
+        <v>Help people understand how to improve</v>
       </c>
       <c r="F32" t="str">
         <v>true</v>
@@ -20375,7 +20535,7 @@
         <v>D</v>
       </c>
       <c r="E33" t="str">
-        <v>The trust, communication, involvement, and effect on people.</v>
+        <v>Link expectations to the wider direction</v>
       </c>
       <c r="F33" t="str">
         <v>true</v>
@@ -20401,7 +20561,7 @@
         <v>A</v>
       </c>
       <c r="E34" t="str">
-        <v>The outcome, owner, decision, and next visible move.</v>
+        <v>Helping people feel supported</v>
       </c>
       <c r="F34" t="str">
         <v>true</v>
@@ -20427,7 +20587,7 @@
         <v>B</v>
       </c>
       <c r="E35" t="str">
-        <v>The structure, sequence, standard, and reliable way of working.</v>
+        <v>Making work feel consistent</v>
       </c>
       <c r="F35" t="str">
         <v>true</v>
@@ -20453,7 +20613,7 @@
         <v>C</v>
       </c>
       <c r="E36" t="str">
-        <v>The future direction, wider meaning, and frame for the choice.</v>
+        <v>Keeping focus on what must be delivered</v>
       </c>
       <c r="F36" t="str">
         <v>true</v>
@@ -20479,7 +20639,7 @@
         <v>D</v>
       </c>
       <c r="E37" t="str">
-        <v>The trust, communication, involvement, and effect on people.</v>
+        <v>Helping people see where things are heading</v>
       </c>
       <c r="F37" t="str">
         <v>true</v>
@@ -20505,7 +20665,7 @@
         <v>A</v>
       </c>
       <c r="E38" t="str">
-        <v>The outcome, owner, decision, and next visible move.</v>
+        <v>Clear about how work should run</v>
       </c>
       <c r="F38" t="str">
         <v>true</v>
@@ -20531,7 +20691,7 @@
         <v>B</v>
       </c>
       <c r="E39" t="str">
-        <v>The structure, sequence, standard, and reliable way of working.</v>
+        <v>Focused on what needs to be delivered</v>
       </c>
       <c r="F39" t="str">
         <v>true</v>
@@ -20557,7 +20717,7 @@
         <v>C</v>
       </c>
       <c r="E40" t="str">
-        <v>The future direction, wider meaning, and frame for the choice.</v>
+        <v>Attentive to what people need</v>
       </c>
       <c r="F40" t="str">
         <v>true</v>
@@ -20583,7 +20743,7 @@
         <v>D</v>
       </c>
       <c r="E41" t="str">
-        <v>The trust, communication, involvement, and effect on people.</v>
+        <v>Focused on where things are heading</v>
       </c>
       <c r="F41" t="str">
         <v>true</v>
@@ -20609,7 +20769,7 @@
         <v>A</v>
       </c>
       <c r="E42" t="str">
-        <v>The outcome, owner, decision, and next visible move.</v>
+        <v>Check what the team needs</v>
       </c>
       <c r="F42" t="str">
         <v>true</v>
@@ -20635,7 +20795,7 @@
         <v>B</v>
       </c>
       <c r="E43" t="str">
-        <v>The structure, sequence, standard, and reliable way of working.</v>
+        <v>Clarify how the work should run</v>
       </c>
       <c r="F43" t="str">
         <v>true</v>
@@ -20661,7 +20821,7 @@
         <v>C</v>
       </c>
       <c r="E44" t="str">
-        <v>The future direction, wider meaning, and frame for the choice.</v>
+        <v>Bring focus back to what must be delivered</v>
       </c>
       <c r="F44" t="str">
         <v>true</v>
@@ -20687,7 +20847,7 @@
         <v>D</v>
       </c>
       <c r="E45" t="str">
-        <v>The trust, communication, involvement, and effect on people.</v>
+        <v>Reconnect the work to the direction</v>
       </c>
       <c r="F45" t="str">
         <v>true</v>
@@ -20713,7 +20873,7 @@
         <v>A</v>
       </c>
       <c r="E46" t="str">
-        <v>The outcome, owner, decision, and next visible move.</v>
+        <v>Keeping the work clearly organised</v>
       </c>
       <c r="F46" t="str">
         <v>true</v>
@@ -20739,7 +20899,7 @@
         <v>B</v>
       </c>
       <c r="E47" t="str">
-        <v>The structure, sequence, standard, and reliable way of working.</v>
+        <v>Making sure the outcome is delivered</v>
       </c>
       <c r="F47" t="str">
         <v>true</v>
@@ -20765,7 +20925,7 @@
         <v>C</v>
       </c>
       <c r="E48" t="str">
-        <v>The future direction, wider meaning, and frame for the choice.</v>
+        <v>Making sure people can keep going</v>
       </c>
       <c r="F48" t="str">
         <v>true</v>
@@ -20791,7 +20951,7 @@
         <v>D</v>
       </c>
       <c r="E49" t="str">
-        <v>The trust, communication, involvement, and effect on people.</v>
+        <v>Keeping choices aligned with direction</v>
       </c>
       <c r="F49" t="str">
         <v>true</v>
@@ -20817,7 +20977,7 @@
         <v>A</v>
       </c>
       <c r="E50" t="str">
-        <v>The outcome, owner, decision, and next visible move.</v>
+        <v>When people are not engaged</v>
       </c>
       <c r="F50" t="str">
         <v>true</v>
@@ -20843,7 +21003,7 @@
         <v>B</v>
       </c>
       <c r="E51" t="str">
-        <v>The structure, sequence, standard, and reliable way of working.</v>
+        <v>When the way of working is unclear</v>
       </c>
       <c r="F51" t="str">
         <v>true</v>
@@ -20869,7 +21029,7 @@
         <v>C</v>
       </c>
       <c r="E52" t="str">
-        <v>The future direction, wider meaning, and frame for the choice.</v>
+        <v>When effort is not producing results</v>
       </c>
       <c r="F52" t="str">
         <v>true</v>
@@ -20895,7 +21055,7 @@
         <v>D</v>
       </c>
       <c r="E53" t="str">
-        <v>The trust, communication, involvement, and effect on people.</v>
+        <v>When the direction is unclear</v>
       </c>
       <c r="F53" t="str">
         <v>true</v>
@@ -20921,7 +21081,7 @@
         <v>A</v>
       </c>
       <c r="E54" t="str">
-        <v>The outcome, owner, decision, and next visible move.</v>
+        <v>The work is clearly organised</v>
       </c>
       <c r="F54" t="str">
         <v>true</v>
@@ -20947,7 +21107,7 @@
         <v>B</v>
       </c>
       <c r="E55" t="str">
-        <v>The structure, sequence, standard, and reliable way of working.</v>
+        <v>Progress is visible and consistent</v>
       </c>
       <c r="F55" t="str">
         <v>true</v>
@@ -20973,7 +21133,7 @@
         <v>C</v>
       </c>
       <c r="E56" t="str">
-        <v>The future direction, wider meaning, and frame for the choice.</v>
+        <v>People feel able to contribute</v>
       </c>
       <c r="F56" t="str">
         <v>true</v>
@@ -20999,7 +21159,7 @@
         <v>D</v>
       </c>
       <c r="E57" t="str">
-        <v>The trust, communication, involvement, and effect on people.</v>
+        <v>The team understands where the work is heading</v>
       </c>
       <c r="F57" t="str">
         <v>true</v>
@@ -21025,7 +21185,7 @@
         <v>A</v>
       </c>
       <c r="E58" t="str">
-        <v>The outcome, owner, decision, and next visible move.</v>
+        <v>People have what they need</v>
       </c>
       <c r="F58" t="str">
         <v>true</v>
@@ -21051,7 +21211,7 @@
         <v>B</v>
       </c>
       <c r="E59" t="str">
-        <v>The structure, sequence, standard, and reliable way of working.</v>
+        <v>The way the work is organised</v>
       </c>
       <c r="F59" t="str">
         <v>true</v>
@@ -21077,7 +21237,7 @@
         <v>C</v>
       </c>
       <c r="E60" t="str">
-        <v>The future direction, wider meaning, and frame for the choice.</v>
+        <v>The outcome that needs to be delivered</v>
       </c>
       <c r="F60" t="str">
         <v>true</v>
@@ -21103,7 +21263,7 @@
         <v>D</v>
       </c>
       <c r="E61" t="str">
-        <v>The trust, communication, involvement, and effect on people.</v>
+        <v>The reason the work matters</v>
       </c>
       <c r="F61" t="str">
         <v>true</v>
@@ -21129,7 +21289,7 @@
         <v>A</v>
       </c>
       <c r="E62" t="str">
-        <v>The outcome, owner, decision, and next visible move.</v>
+        <v>Listen and understand the concern</v>
       </c>
       <c r="F62" t="str">
         <v>true</v>
@@ -21155,7 +21315,7 @@
         <v>B</v>
       </c>
       <c r="E63" t="str">
-        <v>The structure, sequence, standard, and reliable way of working.</v>
+        <v>Clarify how the work should run</v>
       </c>
       <c r="F63" t="str">
         <v>true</v>
@@ -21181,7 +21341,7 @@
         <v>C</v>
       </c>
       <c r="E64" t="str">
-        <v>The future direction, wider meaning, and frame for the choice.</v>
+        <v>Clarify what still needs to be delivered</v>
       </c>
       <c r="F64" t="str">
         <v>true</v>
@@ -21207,7 +21367,7 @@
         <v>D</v>
       </c>
       <c r="E65" t="str">
-        <v>The trust, communication, involvement, and effect on people.</v>
+        <v>Step back and check the direction</v>
       </c>
       <c r="F65" t="str">
         <v>true</v>
@@ -21219,16 +21379,848 @@
         <v>leadership_approach_q16::D</v>
       </c>
     </row>
+    <row r="66">
+      <c r="A66" t="str">
+        <v>leadership_approach</v>
+      </c>
+      <c r="B66" t="str">
+        <v>leadership_approach_q17</v>
+      </c>
+      <c r="C66" t="str">
+        <v>A</v>
+      </c>
+      <c r="D66" t="str">
+        <v>A</v>
+      </c>
+      <c r="E66" t="str">
+        <v>Spend less time checking in with people</v>
+      </c>
+      <c r="F66" t="str">
+        <v>true</v>
+      </c>
+      <c r="G66" t="str">
+        <v>active</v>
+      </c>
+      <c r="H66" t="str">
+        <v>leadership_approach_q17::A</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="str">
+        <v>leadership_approach</v>
+      </c>
+      <c r="B67" t="str">
+        <v>leadership_approach_q17</v>
+      </c>
+      <c r="C67" t="str">
+        <v>B</v>
+      </c>
+      <c r="D67" t="str">
+        <v>B</v>
+      </c>
+      <c r="E67" t="str">
+        <v>Reduce detail around how the work runs</v>
+      </c>
+      <c r="F67" t="str">
+        <v>true</v>
+      </c>
+      <c r="G67" t="str">
+        <v>active</v>
+      </c>
+      <c r="H67" t="str">
+        <v>leadership_approach_q17::B</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="str">
+        <v>leadership_approach</v>
+      </c>
+      <c r="B68" t="str">
+        <v>leadership_approach_q17</v>
+      </c>
+      <c r="C68" t="str">
+        <v>C</v>
+      </c>
+      <c r="D68" t="str">
+        <v>C</v>
+      </c>
+      <c r="E68" t="str">
+        <v>Limit discussion and move the work forward</v>
+      </c>
+      <c r="F68" t="str">
+        <v>true</v>
+      </c>
+      <c r="G68" t="str">
+        <v>active</v>
+      </c>
+      <c r="H68" t="str">
+        <v>leadership_approach_q17::C</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="str">
+        <v>leadership_approach</v>
+      </c>
+      <c r="B69" t="str">
+        <v>leadership_approach_q17</v>
+      </c>
+      <c r="C69" t="str">
+        <v>D</v>
+      </c>
+      <c r="D69" t="str">
+        <v>D</v>
+      </c>
+      <c r="E69" t="str">
+        <v>Spend less time on the wider direction</v>
+      </c>
+      <c r="F69" t="str">
+        <v>true</v>
+      </c>
+      <c r="G69" t="str">
+        <v>active</v>
+      </c>
+      <c r="H69" t="str">
+        <v>leadership_approach_q17::D</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="str">
+        <v>leadership_approach</v>
+      </c>
+      <c r="B70" t="str">
+        <v>leadership_approach_q18</v>
+      </c>
+      <c r="C70" t="str">
+        <v>A</v>
+      </c>
+      <c r="D70" t="str">
+        <v>A</v>
+      </c>
+      <c r="E70" t="str">
+        <v>Whether people are still engaged</v>
+      </c>
+      <c r="F70" t="str">
+        <v>true</v>
+      </c>
+      <c r="G70" t="str">
+        <v>active</v>
+      </c>
+      <c r="H70" t="str">
+        <v>leadership_approach_q18::A</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="str">
+        <v>leadership_approach</v>
+      </c>
+      <c r="B71" t="str">
+        <v>leadership_approach_q18</v>
+      </c>
+      <c r="C71" t="str">
+        <v>B</v>
+      </c>
+      <c r="D71" t="str">
+        <v>B</v>
+      </c>
+      <c r="E71" t="str">
+        <v>Whether the approach is working</v>
+      </c>
+      <c r="F71" t="str">
+        <v>true</v>
+      </c>
+      <c r="G71" t="str">
+        <v>active</v>
+      </c>
+      <c r="H71" t="str">
+        <v>leadership_approach_q18::B</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="str">
+        <v>leadership_approach</v>
+      </c>
+      <c r="B72" t="str">
+        <v>leadership_approach_q18</v>
+      </c>
+      <c r="C72" t="str">
+        <v>C</v>
+      </c>
+      <c r="D72" t="str">
+        <v>C</v>
+      </c>
+      <c r="E72" t="str">
+        <v>Whether progress is visible</v>
+      </c>
+      <c r="F72" t="str">
+        <v>true</v>
+      </c>
+      <c r="G72" t="str">
+        <v>active</v>
+      </c>
+      <c r="H72" t="str">
+        <v>leadership_approach_q18::C</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="str">
+        <v>leadership_approach</v>
+      </c>
+      <c r="B73" t="str">
+        <v>leadership_approach_q18</v>
+      </c>
+      <c r="C73" t="str">
+        <v>D</v>
+      </c>
+      <c r="D73" t="str">
+        <v>D</v>
+      </c>
+      <c r="E73" t="str">
+        <v>Whether the direction is still clear</v>
+      </c>
+      <c r="F73" t="str">
+        <v>true</v>
+      </c>
+      <c r="G73" t="str">
+        <v>active</v>
+      </c>
+      <c r="H73" t="str">
+        <v>leadership_approach_q18::D</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="str">
+        <v>leadership_approach</v>
+      </c>
+      <c r="B74" t="str">
+        <v>leadership_approach_q19</v>
+      </c>
+      <c r="C74" t="str">
+        <v>A</v>
+      </c>
+      <c r="D74" t="str">
+        <v>A</v>
+      </c>
+      <c r="E74" t="str">
+        <v>Make space for concerns to be heard</v>
+      </c>
+      <c r="F74" t="str">
+        <v>true</v>
+      </c>
+      <c r="G74" t="str">
+        <v>active</v>
+      </c>
+      <c r="H74" t="str">
+        <v>leadership_approach_q19::A</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="str">
+        <v>leadership_approach</v>
+      </c>
+      <c r="B75" t="str">
+        <v>leadership_approach_q19</v>
+      </c>
+      <c r="C75" t="str">
+        <v>B</v>
+      </c>
+      <c r="D75" t="str">
+        <v>B</v>
+      </c>
+      <c r="E75" t="str">
+        <v>Clarify what is agreed and what happens next</v>
+      </c>
+      <c r="F75" t="str">
+        <v>true</v>
+      </c>
+      <c r="G75" t="str">
+        <v>active</v>
+      </c>
+      <c r="H75" t="str">
+        <v>leadership_approach_q19::B</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="str">
+        <v>leadership_approach</v>
+      </c>
+      <c r="B76" t="str">
+        <v>leadership_approach_q19</v>
+      </c>
+      <c r="C76" t="str">
+        <v>C</v>
+      </c>
+      <c r="D76" t="str">
+        <v>C</v>
+      </c>
+      <c r="E76" t="str">
+        <v>Bring focus back to the outcome</v>
+      </c>
+      <c r="F76" t="str">
+        <v>true</v>
+      </c>
+      <c r="G76" t="str">
+        <v>active</v>
+      </c>
+      <c r="H76" t="str">
+        <v>leadership_approach_q19::C</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="str">
+        <v>leadership_approach</v>
+      </c>
+      <c r="B77" t="str">
+        <v>leadership_approach_q19</v>
+      </c>
+      <c r="C77" t="str">
+        <v>D</v>
+      </c>
+      <c r="D77" t="str">
+        <v>D</v>
+      </c>
+      <c r="E77" t="str">
+        <v>Reconnect the discussion to the bigger picture</v>
+      </c>
+      <c r="F77" t="str">
+        <v>true</v>
+      </c>
+      <c r="G77" t="str">
+        <v>active</v>
+      </c>
+      <c r="H77" t="str">
+        <v>leadership_approach_q19::D</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="str">
+        <v>leadership_approach</v>
+      </c>
+      <c r="B78" t="str">
+        <v>leadership_approach_q20</v>
+      </c>
+      <c r="C78" t="str">
+        <v>A</v>
+      </c>
+      <c r="D78" t="str">
+        <v>A</v>
+      </c>
+      <c r="E78" t="str">
+        <v>When morale or trust starts to drop</v>
+      </c>
+      <c r="F78" t="str">
+        <v>true</v>
+      </c>
+      <c r="G78" t="str">
+        <v>active</v>
+      </c>
+      <c r="H78" t="str">
+        <v>leadership_approach_q20::A</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="str">
+        <v>leadership_approach</v>
+      </c>
+      <c r="B79" t="str">
+        <v>leadership_approach_q20</v>
+      </c>
+      <c r="C79" t="str">
+        <v>B</v>
+      </c>
+      <c r="D79" t="str">
+        <v>B</v>
+      </c>
+      <c r="E79" t="str">
+        <v>When the work feels disorganised</v>
+      </c>
+      <c r="F79" t="str">
+        <v>true</v>
+      </c>
+      <c r="G79" t="str">
+        <v>active</v>
+      </c>
+      <c r="H79" t="str">
+        <v>leadership_approach_q20::B</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="str">
+        <v>leadership_approach</v>
+      </c>
+      <c r="B80" t="str">
+        <v>leadership_approach_q20</v>
+      </c>
+      <c r="C80" t="str">
+        <v>C</v>
+      </c>
+      <c r="D80" t="str">
+        <v>C</v>
+      </c>
+      <c r="E80" t="str">
+        <v>When work is not producing results</v>
+      </c>
+      <c r="F80" t="str">
+        <v>true</v>
+      </c>
+      <c r="G80" t="str">
+        <v>active</v>
+      </c>
+      <c r="H80" t="str">
+        <v>leadership_approach_q20::C</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="str">
+        <v>leadership_approach</v>
+      </c>
+      <c r="B81" t="str">
+        <v>leadership_approach_q20</v>
+      </c>
+      <c r="C81" t="str">
+        <v>D</v>
+      </c>
+      <c r="D81" t="str">
+        <v>D</v>
+      </c>
+      <c r="E81" t="str">
+        <v>When the direction is unclear</v>
+      </c>
+      <c r="F81" t="str">
+        <v>true</v>
+      </c>
+      <c r="G81" t="str">
+        <v>active</v>
+      </c>
+      <c r="H81" t="str">
+        <v>leadership_approach_q20::D</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="str">
+        <v>leadership_approach</v>
+      </c>
+      <c r="B82" t="str">
+        <v>leadership_approach_q21</v>
+      </c>
+      <c r="C82" t="str">
+        <v>A</v>
+      </c>
+      <c r="D82" t="str">
+        <v>A</v>
+      </c>
+      <c r="E82" t="str">
+        <v>Check what people need</v>
+      </c>
+      <c r="F82" t="str">
+        <v>true</v>
+      </c>
+      <c r="G82" t="str">
+        <v>active</v>
+      </c>
+      <c r="H82" t="str">
+        <v>leadership_approach_q21::A</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="str">
+        <v>leadership_approach</v>
+      </c>
+      <c r="B83" t="str">
+        <v>leadership_approach_q21</v>
+      </c>
+      <c r="C83" t="str">
+        <v>B</v>
+      </c>
+      <c r="D83" t="str">
+        <v>B</v>
+      </c>
+      <c r="E83" t="str">
+        <v>Adjust how the work is running</v>
+      </c>
+      <c r="F83" t="str">
+        <v>true</v>
+      </c>
+      <c r="G83" t="str">
+        <v>active</v>
+      </c>
+      <c r="H83" t="str">
+        <v>leadership_approach_q21::B</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="str">
+        <v>leadership_approach</v>
+      </c>
+      <c r="B84" t="str">
+        <v>leadership_approach_q21</v>
+      </c>
+      <c r="C84" t="str">
+        <v>C</v>
+      </c>
+      <c r="D84" t="str">
+        <v>C</v>
+      </c>
+      <c r="E84" t="str">
+        <v>Focus on the next outcome</v>
+      </c>
+      <c r="F84" t="str">
+        <v>true</v>
+      </c>
+      <c r="G84" t="str">
+        <v>active</v>
+      </c>
+      <c r="H84" t="str">
+        <v>leadership_approach_q21::C</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="str">
+        <v>leadership_approach</v>
+      </c>
+      <c r="B85" t="str">
+        <v>leadership_approach_q21</v>
+      </c>
+      <c r="C85" t="str">
+        <v>D</v>
+      </c>
+      <c r="D85" t="str">
+        <v>D</v>
+      </c>
+      <c r="E85" t="str">
+        <v>Revisit where the work is heading</v>
+      </c>
+      <c r="F85" t="str">
+        <v>true</v>
+      </c>
+      <c r="G85" t="str">
+        <v>active</v>
+      </c>
+      <c r="H85" t="str">
+        <v>leadership_approach_q21::D</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="str">
+        <v>leadership_approach</v>
+      </c>
+      <c r="B86" t="str">
+        <v>leadership_approach_q22</v>
+      </c>
+      <c r="C86" t="str">
+        <v>A</v>
+      </c>
+      <c r="D86" t="str">
+        <v>A</v>
+      </c>
+      <c r="E86" t="str">
+        <v>Who needs to be involved and heard</v>
+      </c>
+      <c r="F86" t="str">
+        <v>true</v>
+      </c>
+      <c r="G86" t="str">
+        <v>active</v>
+      </c>
+      <c r="H86" t="str">
+        <v>leadership_approach_q22::A</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="str">
+        <v>leadership_approach</v>
+      </c>
+      <c r="B87" t="str">
+        <v>leadership_approach_q22</v>
+      </c>
+      <c r="C87" t="str">
+        <v>B</v>
+      </c>
+      <c r="D87" t="str">
+        <v>B</v>
+      </c>
+      <c r="E87" t="str">
+        <v>How the work should run</v>
+      </c>
+      <c r="F87" t="str">
+        <v>true</v>
+      </c>
+      <c r="G87" t="str">
+        <v>active</v>
+      </c>
+      <c r="H87" t="str">
+        <v>leadership_approach_q22::B</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="str">
+        <v>leadership_approach</v>
+      </c>
+      <c r="B88" t="str">
+        <v>leadership_approach_q22</v>
+      </c>
+      <c r="C88" t="str">
+        <v>C</v>
+      </c>
+      <c r="D88" t="str">
+        <v>C</v>
+      </c>
+      <c r="E88" t="str">
+        <v>What needs to be delivered</v>
+      </c>
+      <c r="F88" t="str">
+        <v>true</v>
+      </c>
+      <c r="G88" t="str">
+        <v>active</v>
+      </c>
+      <c r="H88" t="str">
+        <v>leadership_approach_q22::C</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="str">
+        <v>leadership_approach</v>
+      </c>
+      <c r="B89" t="str">
+        <v>leadership_approach_q22</v>
+      </c>
+      <c r="C89" t="str">
+        <v>D</v>
+      </c>
+      <c r="D89" t="str">
+        <v>D</v>
+      </c>
+      <c r="E89" t="str">
+        <v>Where the work is heading</v>
+      </c>
+      <c r="F89" t="str">
+        <v>true</v>
+      </c>
+      <c r="G89" t="str">
+        <v>active</v>
+      </c>
+      <c r="H89" t="str">
+        <v>leadership_approach_q22::D</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="str">
+        <v>leadership_approach</v>
+      </c>
+      <c r="B90" t="str">
+        <v>leadership_approach_q23</v>
+      </c>
+      <c r="C90" t="str">
+        <v>A</v>
+      </c>
+      <c r="D90" t="str">
+        <v>A</v>
+      </c>
+      <c r="E90" t="str">
+        <v>What the people involved need</v>
+      </c>
+      <c r="F90" t="str">
+        <v>true</v>
+      </c>
+      <c r="G90" t="str">
+        <v>active</v>
+      </c>
+      <c r="H90" t="str">
+        <v>leadership_approach_q23::A</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="str">
+        <v>leadership_approach</v>
+      </c>
+      <c r="B91" t="str">
+        <v>leadership_approach_q23</v>
+      </c>
+      <c r="C91" t="str">
+        <v>B</v>
+      </c>
+      <c r="D91" t="str">
+        <v>B</v>
+      </c>
+      <c r="E91" t="str">
+        <v>Where the way of working broke down</v>
+      </c>
+      <c r="F91" t="str">
+        <v>true</v>
+      </c>
+      <c r="G91" t="str">
+        <v>active</v>
+      </c>
+      <c r="H91" t="str">
+        <v>leadership_approach_q23::B</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="str">
+        <v>leadership_approach</v>
+      </c>
+      <c r="B92" t="str">
+        <v>leadership_approach_q23</v>
+      </c>
+      <c r="C92" t="str">
+        <v>C</v>
+      </c>
+      <c r="D92" t="str">
+        <v>C</v>
+      </c>
+      <c r="E92" t="str">
+        <v>What needs to be recovered first</v>
+      </c>
+      <c r="F92" t="str">
+        <v>true</v>
+      </c>
+      <c r="G92" t="str">
+        <v>active</v>
+      </c>
+      <c r="H92" t="str">
+        <v>leadership_approach_q23::C</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="str">
+        <v>leadership_approach</v>
+      </c>
+      <c r="B93" t="str">
+        <v>leadership_approach_q23</v>
+      </c>
+      <c r="C93" t="str">
+        <v>D</v>
+      </c>
+      <c r="D93" t="str">
+        <v>D</v>
+      </c>
+      <c r="E93" t="str">
+        <v>Whether the direction still makes sense</v>
+      </c>
+      <c r="F93" t="str">
+        <v>true</v>
+      </c>
+      <c r="G93" t="str">
+        <v>active</v>
+      </c>
+      <c r="H93" t="str">
+        <v>leadership_approach_q23::D</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="str">
+        <v>leadership_approach</v>
+      </c>
+      <c r="B94" t="str">
+        <v>leadership_approach_q24</v>
+      </c>
+      <c r="C94" t="str">
+        <v>A</v>
+      </c>
+      <c r="D94" t="str">
+        <v>A</v>
+      </c>
+      <c r="E94" t="str">
+        <v>Recognise what people are contributing</v>
+      </c>
+      <c r="F94" t="str">
+        <v>true</v>
+      </c>
+      <c r="G94" t="str">
+        <v>active</v>
+      </c>
+      <c r="H94" t="str">
+        <v>leadership_approach_q24::A</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="str">
+        <v>leadership_approach</v>
+      </c>
+      <c r="B95" t="str">
+        <v>leadership_approach_q24</v>
+      </c>
+      <c r="C95" t="str">
+        <v>B</v>
+      </c>
+      <c r="D95" t="str">
+        <v>B</v>
+      </c>
+      <c r="E95" t="str">
+        <v>Keep the way of working consistent</v>
+      </c>
+      <c r="F95" t="str">
+        <v>true</v>
+      </c>
+      <c r="G95" t="str">
+        <v>active</v>
+      </c>
+      <c r="H95" t="str">
+        <v>leadership_approach_q24::B</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="str">
+        <v>leadership_approach</v>
+      </c>
+      <c r="B96" t="str">
+        <v>leadership_approach_q24</v>
+      </c>
+      <c r="C96" t="str">
+        <v>C</v>
+      </c>
+      <c r="D96" t="str">
+        <v>C</v>
+      </c>
+      <c r="E96" t="str">
+        <v>Set the next outcome to aim for</v>
+      </c>
+      <c r="F96" t="str">
+        <v>true</v>
+      </c>
+      <c r="G96" t="str">
+        <v>active</v>
+      </c>
+      <c r="H96" t="str">
+        <v>leadership_approach_q24::C</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="str">
+        <v>leadership_approach</v>
+      </c>
+      <c r="B97" t="str">
+        <v>leadership_approach_q24</v>
+      </c>
+      <c r="C97" t="str">
+        <v>D</v>
+      </c>
+      <c r="D97" t="str">
+        <v>D</v>
+      </c>
+      <c r="E97" t="str">
+        <v>Keep the work connected to the direction</v>
+      </c>
+      <c r="F97" t="str">
+        <v>true</v>
+      </c>
+      <c r="G97" t="str">
+        <v>active</v>
+      </c>
+      <c r="H97" t="str">
+        <v>leadership_approach_q24::D</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H65"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H97"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G65"/>
+  <dimension ref="A1:G97"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -21267,7 +22259,7 @@
         <v>results</v>
       </c>
       <c r="E2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F2" t="str">
         <v>active</v>
@@ -21287,16 +22279,16 @@
         <v>B</v>
       </c>
       <c r="D3" t="str">
-        <v>process</v>
+        <v>vision</v>
       </c>
       <c r="E3">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F3" t="str">
         <v>active</v>
       </c>
       <c r="G3" t="str">
-        <v>leadership_approach_q01::B::process</v>
+        <v>leadership_approach_q01::B::vision</v>
       </c>
     </row>
     <row r="4">
@@ -21310,16 +22302,16 @@
         <v>C</v>
       </c>
       <c r="D4" t="str">
-        <v>vision</v>
+        <v>process</v>
       </c>
       <c r="E4">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F4" t="str">
         <v>active</v>
       </c>
       <c r="G4" t="str">
-        <v>leadership_approach_q01::C::vision</v>
+        <v>leadership_approach_q01::C::process</v>
       </c>
     </row>
     <row r="5">
@@ -21336,7 +22328,7 @@
         <v>people</v>
       </c>
       <c r="E5">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F5" t="str">
         <v>active</v>
@@ -21356,16 +22348,16 @@
         <v>A</v>
       </c>
       <c r="D6" t="str">
-        <v>results</v>
+        <v>process</v>
       </c>
       <c r="E6">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F6" t="str">
         <v>active</v>
       </c>
       <c r="G6" t="str">
-        <v>leadership_approach_q02::A::results</v>
+        <v>leadership_approach_q02::A::process</v>
       </c>
     </row>
     <row r="7">
@@ -21379,16 +22371,16 @@
         <v>B</v>
       </c>
       <c r="D7" t="str">
-        <v>process</v>
+        <v>results</v>
       </c>
       <c r="E7">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F7" t="str">
         <v>active</v>
       </c>
       <c r="G7" t="str">
-        <v>leadership_approach_q02::B::process</v>
+        <v>leadership_approach_q02::B::results</v>
       </c>
     </row>
     <row r="8">
@@ -21402,16 +22394,16 @@
         <v>C</v>
       </c>
       <c r="D8" t="str">
-        <v>vision</v>
+        <v>people</v>
       </c>
       <c r="E8">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F8" t="str">
         <v>active</v>
       </c>
       <c r="G8" t="str">
-        <v>leadership_approach_q02::C::vision</v>
+        <v>leadership_approach_q02::C::people</v>
       </c>
     </row>
     <row r="9">
@@ -21425,16 +22417,16 @@
         <v>D</v>
       </c>
       <c r="D9" t="str">
-        <v>people</v>
+        <v>vision</v>
       </c>
       <c r="E9">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F9" t="str">
         <v>active</v>
       </c>
       <c r="G9" t="str">
-        <v>leadership_approach_q02::D::people</v>
+        <v>leadership_approach_q02::D::vision</v>
       </c>
     </row>
     <row r="10">
@@ -21448,16 +22440,16 @@
         <v>A</v>
       </c>
       <c r="D10" t="str">
-        <v>results</v>
+        <v>people</v>
       </c>
       <c r="E10">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F10" t="str">
         <v>active</v>
       </c>
       <c r="G10" t="str">
-        <v>leadership_approach_q03::A::results</v>
+        <v>leadership_approach_q03::A::people</v>
       </c>
     </row>
     <row r="11">
@@ -21474,7 +22466,7 @@
         <v>process</v>
       </c>
       <c r="E11">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F11" t="str">
         <v>active</v>
@@ -21494,16 +22486,16 @@
         <v>C</v>
       </c>
       <c r="D12" t="str">
-        <v>vision</v>
+        <v>results</v>
       </c>
       <c r="E12">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F12" t="str">
         <v>active</v>
       </c>
       <c r="G12" t="str">
-        <v>leadership_approach_q03::C::vision</v>
+        <v>leadership_approach_q03::C::results</v>
       </c>
     </row>
     <row r="13">
@@ -21517,16 +22509,16 @@
         <v>D</v>
       </c>
       <c r="D13" t="str">
-        <v>people</v>
+        <v>vision</v>
       </c>
       <c r="E13">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F13" t="str">
         <v>active</v>
       </c>
       <c r="G13" t="str">
-        <v>leadership_approach_q03::D::people</v>
+        <v>leadership_approach_q03::D::vision</v>
       </c>
     </row>
     <row r="14">
@@ -21540,16 +22532,16 @@
         <v>A</v>
       </c>
       <c r="D14" t="str">
-        <v>results</v>
+        <v>process</v>
       </c>
       <c r="E14">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F14" t="str">
         <v>active</v>
       </c>
       <c r="G14" t="str">
-        <v>leadership_approach_q04::A::results</v>
+        <v>leadership_approach_q04::A::process</v>
       </c>
     </row>
     <row r="15">
@@ -21563,16 +22555,16 @@
         <v>B</v>
       </c>
       <c r="D15" t="str">
-        <v>process</v>
+        <v>people</v>
       </c>
       <c r="E15">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F15" t="str">
         <v>active</v>
       </c>
       <c r="G15" t="str">
-        <v>leadership_approach_q04::B::process</v>
+        <v>leadership_approach_q04::B::people</v>
       </c>
     </row>
     <row r="16">
@@ -21586,16 +22578,16 @@
         <v>C</v>
       </c>
       <c r="D16" t="str">
-        <v>vision</v>
+        <v>results</v>
       </c>
       <c r="E16">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F16" t="str">
         <v>active</v>
       </c>
       <c r="G16" t="str">
-        <v>leadership_approach_q04::C::vision</v>
+        <v>leadership_approach_q04::C::results</v>
       </c>
     </row>
     <row r="17">
@@ -21609,16 +22601,16 @@
         <v>D</v>
       </c>
       <c r="D17" t="str">
-        <v>people</v>
+        <v>vision</v>
       </c>
       <c r="E17">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F17" t="str">
         <v>active</v>
       </c>
       <c r="G17" t="str">
-        <v>leadership_approach_q04::D::people</v>
+        <v>leadership_approach_q04::D::vision</v>
       </c>
     </row>
     <row r="18">
@@ -21632,16 +22624,16 @@
         <v>A</v>
       </c>
       <c r="D18" t="str">
-        <v>results</v>
+        <v>people</v>
       </c>
       <c r="E18">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F18" t="str">
         <v>active</v>
       </c>
       <c r="G18" t="str">
-        <v>leadership_approach_q05::A::results</v>
+        <v>leadership_approach_q05::A::people</v>
       </c>
     </row>
     <row r="19">
@@ -21655,16 +22647,16 @@
         <v>B</v>
       </c>
       <c r="D19" t="str">
-        <v>process</v>
+        <v>results</v>
       </c>
       <c r="E19">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F19" t="str">
         <v>active</v>
       </c>
       <c r="G19" t="str">
-        <v>leadership_approach_q05::B::process</v>
+        <v>leadership_approach_q05::B::results</v>
       </c>
     </row>
     <row r="20">
@@ -21678,16 +22670,16 @@
         <v>C</v>
       </c>
       <c r="D20" t="str">
-        <v>vision</v>
+        <v>process</v>
       </c>
       <c r="E20">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F20" t="str">
         <v>active</v>
       </c>
       <c r="G20" t="str">
-        <v>leadership_approach_q05::C::vision</v>
+        <v>leadership_approach_q05::C::process</v>
       </c>
     </row>
     <row r="21">
@@ -21701,16 +22693,16 @@
         <v>D</v>
       </c>
       <c r="D21" t="str">
-        <v>people</v>
+        <v>vision</v>
       </c>
       <c r="E21">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F21" t="str">
         <v>active</v>
       </c>
       <c r="G21" t="str">
-        <v>leadership_approach_q05::D::people</v>
+        <v>leadership_approach_q05::D::vision</v>
       </c>
     </row>
     <row r="22">
@@ -21724,16 +22716,16 @@
         <v>A</v>
       </c>
       <c r="D22" t="str">
-        <v>results</v>
+        <v>vision</v>
       </c>
       <c r="E22">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F22" t="str">
         <v>active</v>
       </c>
       <c r="G22" t="str">
-        <v>leadership_approach_q06::A::results</v>
+        <v>leadership_approach_q06::A::vision</v>
       </c>
     </row>
     <row r="23">
@@ -21750,7 +22742,7 @@
         <v>process</v>
       </c>
       <c r="E23">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F23" t="str">
         <v>active</v>
@@ -21770,16 +22762,16 @@
         <v>C</v>
       </c>
       <c r="D24" t="str">
-        <v>vision</v>
+        <v>results</v>
       </c>
       <c r="E24">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F24" t="str">
         <v>active</v>
       </c>
       <c r="G24" t="str">
-        <v>leadership_approach_q06::C::vision</v>
+        <v>leadership_approach_q06::C::results</v>
       </c>
     </row>
     <row r="25">
@@ -21796,7 +22788,7 @@
         <v>people</v>
       </c>
       <c r="E25">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F25" t="str">
         <v>active</v>
@@ -21816,16 +22808,16 @@
         <v>A</v>
       </c>
       <c r="D26" t="str">
-        <v>results</v>
+        <v>people</v>
       </c>
       <c r="E26">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F26" t="str">
         <v>active</v>
       </c>
       <c r="G26" t="str">
-        <v>leadership_approach_q07::A::results</v>
+        <v>leadership_approach_q07::A::people</v>
       </c>
     </row>
     <row r="27">
@@ -21842,7 +22834,7 @@
         <v>process</v>
       </c>
       <c r="E27">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F27" t="str">
         <v>active</v>
@@ -21862,16 +22854,16 @@
         <v>C</v>
       </c>
       <c r="D28" t="str">
-        <v>vision</v>
+        <v>results</v>
       </c>
       <c r="E28">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F28" t="str">
         <v>active</v>
       </c>
       <c r="G28" t="str">
-        <v>leadership_approach_q07::C::vision</v>
+        <v>leadership_approach_q07::C::results</v>
       </c>
     </row>
     <row r="29">
@@ -21885,16 +22877,16 @@
         <v>D</v>
       </c>
       <c r="D29" t="str">
-        <v>people</v>
+        <v>vision</v>
       </c>
       <c r="E29">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F29" t="str">
         <v>active</v>
       </c>
       <c r="G29" t="str">
-        <v>leadership_approach_q07::D::people</v>
+        <v>leadership_approach_q07::D::vision</v>
       </c>
     </row>
     <row r="30">
@@ -21908,16 +22900,16 @@
         <v>A</v>
       </c>
       <c r="D30" t="str">
-        <v>results</v>
+        <v>process</v>
       </c>
       <c r="E30">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F30" t="str">
         <v>active</v>
       </c>
       <c r="G30" t="str">
-        <v>leadership_approach_q08::A::results</v>
+        <v>leadership_approach_q08::A::process</v>
       </c>
     </row>
     <row r="31">
@@ -21931,16 +22923,16 @@
         <v>B</v>
       </c>
       <c r="D31" t="str">
-        <v>process</v>
+        <v>results</v>
       </c>
       <c r="E31">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F31" t="str">
         <v>active</v>
       </c>
       <c r="G31" t="str">
-        <v>leadership_approach_q08::B::process</v>
+        <v>leadership_approach_q08::B::results</v>
       </c>
     </row>
     <row r="32">
@@ -21954,16 +22946,16 @@
         <v>C</v>
       </c>
       <c r="D32" t="str">
-        <v>vision</v>
+        <v>people</v>
       </c>
       <c r="E32">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F32" t="str">
         <v>active</v>
       </c>
       <c r="G32" t="str">
-        <v>leadership_approach_q08::C::vision</v>
+        <v>leadership_approach_q08::C::people</v>
       </c>
     </row>
     <row r="33">
@@ -21977,16 +22969,16 @@
         <v>D</v>
       </c>
       <c r="D33" t="str">
-        <v>people</v>
+        <v>vision</v>
       </c>
       <c r="E33">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F33" t="str">
         <v>active</v>
       </c>
       <c r="G33" t="str">
-        <v>leadership_approach_q08::D::people</v>
+        <v>leadership_approach_q08::D::vision</v>
       </c>
     </row>
     <row r="34">
@@ -22000,16 +22992,16 @@
         <v>A</v>
       </c>
       <c r="D34" t="str">
-        <v>results</v>
+        <v>people</v>
       </c>
       <c r="E34">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F34" t="str">
         <v>active</v>
       </c>
       <c r="G34" t="str">
-        <v>leadership_approach_q09::A::results</v>
+        <v>leadership_approach_q09::A::people</v>
       </c>
     </row>
     <row r="35">
@@ -22026,7 +23018,7 @@
         <v>process</v>
       </c>
       <c r="E35">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F35" t="str">
         <v>active</v>
@@ -22046,16 +23038,16 @@
         <v>C</v>
       </c>
       <c r="D36" t="str">
-        <v>vision</v>
+        <v>results</v>
       </c>
       <c r="E36">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F36" t="str">
         <v>active</v>
       </c>
       <c r="G36" t="str">
-        <v>leadership_approach_q09::C::vision</v>
+        <v>leadership_approach_q09::C::results</v>
       </c>
     </row>
     <row r="37">
@@ -22069,16 +23061,16 @@
         <v>D</v>
       </c>
       <c r="D37" t="str">
-        <v>people</v>
+        <v>vision</v>
       </c>
       <c r="E37">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F37" t="str">
         <v>active</v>
       </c>
       <c r="G37" t="str">
-        <v>leadership_approach_q09::D::people</v>
+        <v>leadership_approach_q09::D::vision</v>
       </c>
     </row>
     <row r="38">
@@ -22092,16 +23084,16 @@
         <v>A</v>
       </c>
       <c r="D38" t="str">
-        <v>results</v>
+        <v>process</v>
       </c>
       <c r="E38">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F38" t="str">
         <v>active</v>
       </c>
       <c r="G38" t="str">
-        <v>leadership_approach_q10::A::results</v>
+        <v>leadership_approach_q10::A::process</v>
       </c>
     </row>
     <row r="39">
@@ -22115,16 +23107,16 @@
         <v>B</v>
       </c>
       <c r="D39" t="str">
-        <v>process</v>
+        <v>results</v>
       </c>
       <c r="E39">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F39" t="str">
         <v>active</v>
       </c>
       <c r="G39" t="str">
-        <v>leadership_approach_q10::B::process</v>
+        <v>leadership_approach_q10::B::results</v>
       </c>
     </row>
     <row r="40">
@@ -22138,16 +23130,16 @@
         <v>C</v>
       </c>
       <c r="D40" t="str">
-        <v>vision</v>
+        <v>people</v>
       </c>
       <c r="E40">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F40" t="str">
         <v>active</v>
       </c>
       <c r="G40" t="str">
-        <v>leadership_approach_q10::C::vision</v>
+        <v>leadership_approach_q10::C::people</v>
       </c>
     </row>
     <row r="41">
@@ -22161,16 +23153,16 @@
         <v>D</v>
       </c>
       <c r="D41" t="str">
-        <v>people</v>
+        <v>vision</v>
       </c>
       <c r="E41">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F41" t="str">
         <v>active</v>
       </c>
       <c r="G41" t="str">
-        <v>leadership_approach_q10::D::people</v>
+        <v>leadership_approach_q10::D::vision</v>
       </c>
     </row>
     <row r="42">
@@ -22184,16 +23176,16 @@
         <v>A</v>
       </c>
       <c r="D42" t="str">
-        <v>results</v>
+        <v>people</v>
       </c>
       <c r="E42">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F42" t="str">
         <v>active</v>
       </c>
       <c r="G42" t="str">
-        <v>leadership_approach_q11::A::results</v>
+        <v>leadership_approach_q11::A::people</v>
       </c>
     </row>
     <row r="43">
@@ -22210,7 +23202,7 @@
         <v>process</v>
       </c>
       <c r="E43">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F43" t="str">
         <v>active</v>
@@ -22230,16 +23222,16 @@
         <v>C</v>
       </c>
       <c r="D44" t="str">
-        <v>vision</v>
+        <v>results</v>
       </c>
       <c r="E44">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F44" t="str">
         <v>active</v>
       </c>
       <c r="G44" t="str">
-        <v>leadership_approach_q11::C::vision</v>
+        <v>leadership_approach_q11::C::results</v>
       </c>
     </row>
     <row r="45">
@@ -22253,16 +23245,16 @@
         <v>D</v>
       </c>
       <c r="D45" t="str">
-        <v>people</v>
+        <v>vision</v>
       </c>
       <c r="E45">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F45" t="str">
         <v>active</v>
       </c>
       <c r="G45" t="str">
-        <v>leadership_approach_q11::D::people</v>
+        <v>leadership_approach_q11::D::vision</v>
       </c>
     </row>
     <row r="46">
@@ -22276,16 +23268,16 @@
         <v>A</v>
       </c>
       <c r="D46" t="str">
-        <v>results</v>
+        <v>process</v>
       </c>
       <c r="E46">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F46" t="str">
         <v>active</v>
       </c>
       <c r="G46" t="str">
-        <v>leadership_approach_q12::A::results</v>
+        <v>leadership_approach_q12::A::process</v>
       </c>
     </row>
     <row r="47">
@@ -22299,16 +23291,16 @@
         <v>B</v>
       </c>
       <c r="D47" t="str">
-        <v>process</v>
+        <v>results</v>
       </c>
       <c r="E47">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F47" t="str">
         <v>active</v>
       </c>
       <c r="G47" t="str">
-        <v>leadership_approach_q12::B::process</v>
+        <v>leadership_approach_q12::B::results</v>
       </c>
     </row>
     <row r="48">
@@ -22322,16 +23314,16 @@
         <v>C</v>
       </c>
       <c r="D48" t="str">
-        <v>vision</v>
+        <v>people</v>
       </c>
       <c r="E48">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F48" t="str">
         <v>active</v>
       </c>
       <c r="G48" t="str">
-        <v>leadership_approach_q12::C::vision</v>
+        <v>leadership_approach_q12::C::people</v>
       </c>
     </row>
     <row r="49">
@@ -22345,16 +23337,16 @@
         <v>D</v>
       </c>
       <c r="D49" t="str">
-        <v>people</v>
+        <v>vision</v>
       </c>
       <c r="E49">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F49" t="str">
         <v>active</v>
       </c>
       <c r="G49" t="str">
-        <v>leadership_approach_q12::D::people</v>
+        <v>leadership_approach_q12::D::vision</v>
       </c>
     </row>
     <row r="50">
@@ -22368,16 +23360,16 @@
         <v>A</v>
       </c>
       <c r="D50" t="str">
-        <v>results</v>
+        <v>people</v>
       </c>
       <c r="E50">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F50" t="str">
         <v>active</v>
       </c>
       <c r="G50" t="str">
-        <v>leadership_approach_q13::A::results</v>
+        <v>leadership_approach_q13::A::people</v>
       </c>
     </row>
     <row r="51">
@@ -22394,7 +23386,7 @@
         <v>process</v>
       </c>
       <c r="E51">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F51" t="str">
         <v>active</v>
@@ -22414,16 +23406,16 @@
         <v>C</v>
       </c>
       <c r="D52" t="str">
-        <v>vision</v>
+        <v>results</v>
       </c>
       <c r="E52">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F52" t="str">
         <v>active</v>
       </c>
       <c r="G52" t="str">
-        <v>leadership_approach_q13::C::vision</v>
+        <v>leadership_approach_q13::C::results</v>
       </c>
     </row>
     <row r="53">
@@ -22437,16 +23429,16 @@
         <v>D</v>
       </c>
       <c r="D53" t="str">
-        <v>people</v>
+        <v>vision</v>
       </c>
       <c r="E53">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F53" t="str">
         <v>active</v>
       </c>
       <c r="G53" t="str">
-        <v>leadership_approach_q13::D::people</v>
+        <v>leadership_approach_q13::D::vision</v>
       </c>
     </row>
     <row r="54">
@@ -22460,16 +23452,16 @@
         <v>A</v>
       </c>
       <c r="D54" t="str">
-        <v>results</v>
+        <v>process</v>
       </c>
       <c r="E54">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F54" t="str">
         <v>active</v>
       </c>
       <c r="G54" t="str">
-        <v>leadership_approach_q14::A::results</v>
+        <v>leadership_approach_q14::A::process</v>
       </c>
     </row>
     <row r="55">
@@ -22483,16 +23475,16 @@
         <v>B</v>
       </c>
       <c r="D55" t="str">
-        <v>process</v>
+        <v>results</v>
       </c>
       <c r="E55">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F55" t="str">
         <v>active</v>
       </c>
       <c r="G55" t="str">
-        <v>leadership_approach_q14::B::process</v>
+        <v>leadership_approach_q14::B::results</v>
       </c>
     </row>
     <row r="56">
@@ -22506,16 +23498,16 @@
         <v>C</v>
       </c>
       <c r="D56" t="str">
-        <v>vision</v>
+        <v>people</v>
       </c>
       <c r="E56">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F56" t="str">
         <v>active</v>
       </c>
       <c r="G56" t="str">
-        <v>leadership_approach_q14::C::vision</v>
+        <v>leadership_approach_q14::C::people</v>
       </c>
     </row>
     <row r="57">
@@ -22529,16 +23521,16 @@
         <v>D</v>
       </c>
       <c r="D57" t="str">
-        <v>people</v>
+        <v>vision</v>
       </c>
       <c r="E57">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F57" t="str">
         <v>active</v>
       </c>
       <c r="G57" t="str">
-        <v>leadership_approach_q14::D::people</v>
+        <v>leadership_approach_q14::D::vision</v>
       </c>
     </row>
     <row r="58">
@@ -22552,16 +23544,16 @@
         <v>A</v>
       </c>
       <c r="D58" t="str">
-        <v>results</v>
+        <v>people</v>
       </c>
       <c r="E58">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F58" t="str">
         <v>active</v>
       </c>
       <c r="G58" t="str">
-        <v>leadership_approach_q15::A::results</v>
+        <v>leadership_approach_q15::A::people</v>
       </c>
     </row>
     <row r="59">
@@ -22578,7 +23570,7 @@
         <v>process</v>
       </c>
       <c r="E59">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F59" t="str">
         <v>active</v>
@@ -22598,16 +23590,16 @@
         <v>C</v>
       </c>
       <c r="D60" t="str">
-        <v>vision</v>
+        <v>results</v>
       </c>
       <c r="E60">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F60" t="str">
         <v>active</v>
       </c>
       <c r="G60" t="str">
-        <v>leadership_approach_q15::C::vision</v>
+        <v>leadership_approach_q15::C::results</v>
       </c>
     </row>
     <row r="61">
@@ -22621,16 +23613,16 @@
         <v>D</v>
       </c>
       <c r="D61" t="str">
-        <v>people</v>
+        <v>vision</v>
       </c>
       <c r="E61">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F61" t="str">
         <v>active</v>
       </c>
       <c r="G61" t="str">
-        <v>leadership_approach_q15::D::people</v>
+        <v>leadership_approach_q15::D::vision</v>
       </c>
     </row>
     <row r="62">
@@ -22644,16 +23636,16 @@
         <v>A</v>
       </c>
       <c r="D62" t="str">
-        <v>results</v>
+        <v>people</v>
       </c>
       <c r="E62">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F62" t="str">
         <v>active</v>
       </c>
       <c r="G62" t="str">
-        <v>leadership_approach_q16::A::results</v>
+        <v>leadership_approach_q16::A::people</v>
       </c>
     </row>
     <row r="63">
@@ -22670,7 +23662,7 @@
         <v>process</v>
       </c>
       <c r="E63">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F63" t="str">
         <v>active</v>
@@ -22690,16 +23682,16 @@
         <v>C</v>
       </c>
       <c r="D64" t="str">
-        <v>vision</v>
+        <v>results</v>
       </c>
       <c r="E64">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F64" t="str">
         <v>active</v>
       </c>
       <c r="G64" t="str">
-        <v>leadership_approach_q16::C::vision</v>
+        <v>leadership_approach_q16::C::results</v>
       </c>
     </row>
     <row r="65">
@@ -22713,21 +23705,757 @@
         <v>D</v>
       </c>
       <c r="D65" t="str">
-        <v>people</v>
+        <v>vision</v>
       </c>
       <c r="E65">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F65" t="str">
         <v>active</v>
       </c>
       <c r="G65" t="str">
-        <v>leadership_approach_q16::D::people</v>
+        <v>leadership_approach_q16::D::vision</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="str">
+        <v>leadership_approach</v>
+      </c>
+      <c r="B66" t="str">
+        <v>leadership_approach_q17</v>
+      </c>
+      <c r="C66" t="str">
+        <v>A</v>
+      </c>
+      <c r="D66" t="str">
+        <v>people</v>
+      </c>
+      <c r="E66">
+        <v>1</v>
+      </c>
+      <c r="F66" t="str">
+        <v>active</v>
+      </c>
+      <c r="G66" t="str">
+        <v>leadership_approach_q17::A::people</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="str">
+        <v>leadership_approach</v>
+      </c>
+      <c r="B67" t="str">
+        <v>leadership_approach_q17</v>
+      </c>
+      <c r="C67" t="str">
+        <v>B</v>
+      </c>
+      <c r="D67" t="str">
+        <v>process</v>
+      </c>
+      <c r="E67">
+        <v>1</v>
+      </c>
+      <c r="F67" t="str">
+        <v>active</v>
+      </c>
+      <c r="G67" t="str">
+        <v>leadership_approach_q17::B::process</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="str">
+        <v>leadership_approach</v>
+      </c>
+      <c r="B68" t="str">
+        <v>leadership_approach_q17</v>
+      </c>
+      <c r="C68" t="str">
+        <v>C</v>
+      </c>
+      <c r="D68" t="str">
+        <v>results</v>
+      </c>
+      <c r="E68">
+        <v>1</v>
+      </c>
+      <c r="F68" t="str">
+        <v>active</v>
+      </c>
+      <c r="G68" t="str">
+        <v>leadership_approach_q17::C::results</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="str">
+        <v>leadership_approach</v>
+      </c>
+      <c r="B69" t="str">
+        <v>leadership_approach_q17</v>
+      </c>
+      <c r="C69" t="str">
+        <v>D</v>
+      </c>
+      <c r="D69" t="str">
+        <v>vision</v>
+      </c>
+      <c r="E69">
+        <v>1</v>
+      </c>
+      <c r="F69" t="str">
+        <v>active</v>
+      </c>
+      <c r="G69" t="str">
+        <v>leadership_approach_q17::D::vision</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="str">
+        <v>leadership_approach</v>
+      </c>
+      <c r="B70" t="str">
+        <v>leadership_approach_q18</v>
+      </c>
+      <c r="C70" t="str">
+        <v>A</v>
+      </c>
+      <c r="D70" t="str">
+        <v>people</v>
+      </c>
+      <c r="E70">
+        <v>1</v>
+      </c>
+      <c r="F70" t="str">
+        <v>active</v>
+      </c>
+      <c r="G70" t="str">
+        <v>leadership_approach_q18::A::people</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="str">
+        <v>leadership_approach</v>
+      </c>
+      <c r="B71" t="str">
+        <v>leadership_approach_q18</v>
+      </c>
+      <c r="C71" t="str">
+        <v>B</v>
+      </c>
+      <c r="D71" t="str">
+        <v>process</v>
+      </c>
+      <c r="E71">
+        <v>1</v>
+      </c>
+      <c r="F71" t="str">
+        <v>active</v>
+      </c>
+      <c r="G71" t="str">
+        <v>leadership_approach_q18::B::process</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="str">
+        <v>leadership_approach</v>
+      </c>
+      <c r="B72" t="str">
+        <v>leadership_approach_q18</v>
+      </c>
+      <c r="C72" t="str">
+        <v>C</v>
+      </c>
+      <c r="D72" t="str">
+        <v>results</v>
+      </c>
+      <c r="E72">
+        <v>1</v>
+      </c>
+      <c r="F72" t="str">
+        <v>active</v>
+      </c>
+      <c r="G72" t="str">
+        <v>leadership_approach_q18::C::results</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="str">
+        <v>leadership_approach</v>
+      </c>
+      <c r="B73" t="str">
+        <v>leadership_approach_q18</v>
+      </c>
+      <c r="C73" t="str">
+        <v>D</v>
+      </c>
+      <c r="D73" t="str">
+        <v>vision</v>
+      </c>
+      <c r="E73">
+        <v>1</v>
+      </c>
+      <c r="F73" t="str">
+        <v>active</v>
+      </c>
+      <c r="G73" t="str">
+        <v>leadership_approach_q18::D::vision</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="str">
+        <v>leadership_approach</v>
+      </c>
+      <c r="B74" t="str">
+        <v>leadership_approach_q19</v>
+      </c>
+      <c r="C74" t="str">
+        <v>A</v>
+      </c>
+      <c r="D74" t="str">
+        <v>people</v>
+      </c>
+      <c r="E74">
+        <v>1</v>
+      </c>
+      <c r="F74" t="str">
+        <v>active</v>
+      </c>
+      <c r="G74" t="str">
+        <v>leadership_approach_q19::A::people</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="str">
+        <v>leadership_approach</v>
+      </c>
+      <c r="B75" t="str">
+        <v>leadership_approach_q19</v>
+      </c>
+      <c r="C75" t="str">
+        <v>B</v>
+      </c>
+      <c r="D75" t="str">
+        <v>process</v>
+      </c>
+      <c r="E75">
+        <v>1</v>
+      </c>
+      <c r="F75" t="str">
+        <v>active</v>
+      </c>
+      <c r="G75" t="str">
+        <v>leadership_approach_q19::B::process</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="str">
+        <v>leadership_approach</v>
+      </c>
+      <c r="B76" t="str">
+        <v>leadership_approach_q19</v>
+      </c>
+      <c r="C76" t="str">
+        <v>C</v>
+      </c>
+      <c r="D76" t="str">
+        <v>results</v>
+      </c>
+      <c r="E76">
+        <v>1</v>
+      </c>
+      <c r="F76" t="str">
+        <v>active</v>
+      </c>
+      <c r="G76" t="str">
+        <v>leadership_approach_q19::C::results</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="str">
+        <v>leadership_approach</v>
+      </c>
+      <c r="B77" t="str">
+        <v>leadership_approach_q19</v>
+      </c>
+      <c r="C77" t="str">
+        <v>D</v>
+      </c>
+      <c r="D77" t="str">
+        <v>vision</v>
+      </c>
+      <c r="E77">
+        <v>1</v>
+      </c>
+      <c r="F77" t="str">
+        <v>active</v>
+      </c>
+      <c r="G77" t="str">
+        <v>leadership_approach_q19::D::vision</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="str">
+        <v>leadership_approach</v>
+      </c>
+      <c r="B78" t="str">
+        <v>leadership_approach_q20</v>
+      </c>
+      <c r="C78" t="str">
+        <v>A</v>
+      </c>
+      <c r="D78" t="str">
+        <v>people</v>
+      </c>
+      <c r="E78">
+        <v>1</v>
+      </c>
+      <c r="F78" t="str">
+        <v>active</v>
+      </c>
+      <c r="G78" t="str">
+        <v>leadership_approach_q20::A::people</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="str">
+        <v>leadership_approach</v>
+      </c>
+      <c r="B79" t="str">
+        <v>leadership_approach_q20</v>
+      </c>
+      <c r="C79" t="str">
+        <v>B</v>
+      </c>
+      <c r="D79" t="str">
+        <v>process</v>
+      </c>
+      <c r="E79">
+        <v>1</v>
+      </c>
+      <c r="F79" t="str">
+        <v>active</v>
+      </c>
+      <c r="G79" t="str">
+        <v>leadership_approach_q20::B::process</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="str">
+        <v>leadership_approach</v>
+      </c>
+      <c r="B80" t="str">
+        <v>leadership_approach_q20</v>
+      </c>
+      <c r="C80" t="str">
+        <v>C</v>
+      </c>
+      <c r="D80" t="str">
+        <v>results</v>
+      </c>
+      <c r="E80">
+        <v>1</v>
+      </c>
+      <c r="F80" t="str">
+        <v>active</v>
+      </c>
+      <c r="G80" t="str">
+        <v>leadership_approach_q20::C::results</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="str">
+        <v>leadership_approach</v>
+      </c>
+      <c r="B81" t="str">
+        <v>leadership_approach_q20</v>
+      </c>
+      <c r="C81" t="str">
+        <v>D</v>
+      </c>
+      <c r="D81" t="str">
+        <v>vision</v>
+      </c>
+      <c r="E81">
+        <v>1</v>
+      </c>
+      <c r="F81" t="str">
+        <v>active</v>
+      </c>
+      <c r="G81" t="str">
+        <v>leadership_approach_q20::D::vision</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="str">
+        <v>leadership_approach</v>
+      </c>
+      <c r="B82" t="str">
+        <v>leadership_approach_q21</v>
+      </c>
+      <c r="C82" t="str">
+        <v>A</v>
+      </c>
+      <c r="D82" t="str">
+        <v>people</v>
+      </c>
+      <c r="E82">
+        <v>1</v>
+      </c>
+      <c r="F82" t="str">
+        <v>active</v>
+      </c>
+      <c r="G82" t="str">
+        <v>leadership_approach_q21::A::people</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="str">
+        <v>leadership_approach</v>
+      </c>
+      <c r="B83" t="str">
+        <v>leadership_approach_q21</v>
+      </c>
+      <c r="C83" t="str">
+        <v>B</v>
+      </c>
+      <c r="D83" t="str">
+        <v>process</v>
+      </c>
+      <c r="E83">
+        <v>1</v>
+      </c>
+      <c r="F83" t="str">
+        <v>active</v>
+      </c>
+      <c r="G83" t="str">
+        <v>leadership_approach_q21::B::process</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="str">
+        <v>leadership_approach</v>
+      </c>
+      <c r="B84" t="str">
+        <v>leadership_approach_q21</v>
+      </c>
+      <c r="C84" t="str">
+        <v>C</v>
+      </c>
+      <c r="D84" t="str">
+        <v>results</v>
+      </c>
+      <c r="E84">
+        <v>1</v>
+      </c>
+      <c r="F84" t="str">
+        <v>active</v>
+      </c>
+      <c r="G84" t="str">
+        <v>leadership_approach_q21::C::results</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="str">
+        <v>leadership_approach</v>
+      </c>
+      <c r="B85" t="str">
+        <v>leadership_approach_q21</v>
+      </c>
+      <c r="C85" t="str">
+        <v>D</v>
+      </c>
+      <c r="D85" t="str">
+        <v>vision</v>
+      </c>
+      <c r="E85">
+        <v>1</v>
+      </c>
+      <c r="F85" t="str">
+        <v>active</v>
+      </c>
+      <c r="G85" t="str">
+        <v>leadership_approach_q21::D::vision</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="str">
+        <v>leadership_approach</v>
+      </c>
+      <c r="B86" t="str">
+        <v>leadership_approach_q22</v>
+      </c>
+      <c r="C86" t="str">
+        <v>A</v>
+      </c>
+      <c r="D86" t="str">
+        <v>people</v>
+      </c>
+      <c r="E86">
+        <v>1</v>
+      </c>
+      <c r="F86" t="str">
+        <v>active</v>
+      </c>
+      <c r="G86" t="str">
+        <v>leadership_approach_q22::A::people</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="str">
+        <v>leadership_approach</v>
+      </c>
+      <c r="B87" t="str">
+        <v>leadership_approach_q22</v>
+      </c>
+      <c r="C87" t="str">
+        <v>B</v>
+      </c>
+      <c r="D87" t="str">
+        <v>process</v>
+      </c>
+      <c r="E87">
+        <v>1</v>
+      </c>
+      <c r="F87" t="str">
+        <v>active</v>
+      </c>
+      <c r="G87" t="str">
+        <v>leadership_approach_q22::B::process</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="str">
+        <v>leadership_approach</v>
+      </c>
+      <c r="B88" t="str">
+        <v>leadership_approach_q22</v>
+      </c>
+      <c r="C88" t="str">
+        <v>C</v>
+      </c>
+      <c r="D88" t="str">
+        <v>results</v>
+      </c>
+      <c r="E88">
+        <v>1</v>
+      </c>
+      <c r="F88" t="str">
+        <v>active</v>
+      </c>
+      <c r="G88" t="str">
+        <v>leadership_approach_q22::C::results</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="str">
+        <v>leadership_approach</v>
+      </c>
+      <c r="B89" t="str">
+        <v>leadership_approach_q22</v>
+      </c>
+      <c r="C89" t="str">
+        <v>D</v>
+      </c>
+      <c r="D89" t="str">
+        <v>vision</v>
+      </c>
+      <c r="E89">
+        <v>1</v>
+      </c>
+      <c r="F89" t="str">
+        <v>active</v>
+      </c>
+      <c r="G89" t="str">
+        <v>leadership_approach_q22::D::vision</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="str">
+        <v>leadership_approach</v>
+      </c>
+      <c r="B90" t="str">
+        <v>leadership_approach_q23</v>
+      </c>
+      <c r="C90" t="str">
+        <v>A</v>
+      </c>
+      <c r="D90" t="str">
+        <v>people</v>
+      </c>
+      <c r="E90">
+        <v>1</v>
+      </c>
+      <c r="F90" t="str">
+        <v>active</v>
+      </c>
+      <c r="G90" t="str">
+        <v>leadership_approach_q23::A::people</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="str">
+        <v>leadership_approach</v>
+      </c>
+      <c r="B91" t="str">
+        <v>leadership_approach_q23</v>
+      </c>
+      <c r="C91" t="str">
+        <v>B</v>
+      </c>
+      <c r="D91" t="str">
+        <v>process</v>
+      </c>
+      <c r="E91">
+        <v>1</v>
+      </c>
+      <c r="F91" t="str">
+        <v>active</v>
+      </c>
+      <c r="G91" t="str">
+        <v>leadership_approach_q23::B::process</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="str">
+        <v>leadership_approach</v>
+      </c>
+      <c r="B92" t="str">
+        <v>leadership_approach_q23</v>
+      </c>
+      <c r="C92" t="str">
+        <v>C</v>
+      </c>
+      <c r="D92" t="str">
+        <v>results</v>
+      </c>
+      <c r="E92">
+        <v>1</v>
+      </c>
+      <c r="F92" t="str">
+        <v>active</v>
+      </c>
+      <c r="G92" t="str">
+        <v>leadership_approach_q23::C::results</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="str">
+        <v>leadership_approach</v>
+      </c>
+      <c r="B93" t="str">
+        <v>leadership_approach_q23</v>
+      </c>
+      <c r="C93" t="str">
+        <v>D</v>
+      </c>
+      <c r="D93" t="str">
+        <v>vision</v>
+      </c>
+      <c r="E93">
+        <v>1</v>
+      </c>
+      <c r="F93" t="str">
+        <v>active</v>
+      </c>
+      <c r="G93" t="str">
+        <v>leadership_approach_q23::D::vision</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="str">
+        <v>leadership_approach</v>
+      </c>
+      <c r="B94" t="str">
+        <v>leadership_approach_q24</v>
+      </c>
+      <c r="C94" t="str">
+        <v>A</v>
+      </c>
+      <c r="D94" t="str">
+        <v>people</v>
+      </c>
+      <c r="E94">
+        <v>1</v>
+      </c>
+      <c r="F94" t="str">
+        <v>active</v>
+      </c>
+      <c r="G94" t="str">
+        <v>leadership_approach_q24::A::people</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="str">
+        <v>leadership_approach</v>
+      </c>
+      <c r="B95" t="str">
+        <v>leadership_approach_q24</v>
+      </c>
+      <c r="C95" t="str">
+        <v>B</v>
+      </c>
+      <c r="D95" t="str">
+        <v>process</v>
+      </c>
+      <c r="E95">
+        <v>1</v>
+      </c>
+      <c r="F95" t="str">
+        <v>active</v>
+      </c>
+      <c r="G95" t="str">
+        <v>leadership_approach_q24::B::process</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="str">
+        <v>leadership_approach</v>
+      </c>
+      <c r="B96" t="str">
+        <v>leadership_approach_q24</v>
+      </c>
+      <c r="C96" t="str">
+        <v>C</v>
+      </c>
+      <c r="D96" t="str">
+        <v>results</v>
+      </c>
+      <c r="E96">
+        <v>1</v>
+      </c>
+      <c r="F96" t="str">
+        <v>active</v>
+      </c>
+      <c r="G96" t="str">
+        <v>leadership_approach_q24::C::results</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="str">
+        <v>leadership_approach</v>
+      </c>
+      <c r="B97" t="str">
+        <v>leadership_approach_q24</v>
+      </c>
+      <c r="C97" t="str">
+        <v>D</v>
+      </c>
+      <c r="D97" t="str">
+        <v>vision</v>
+      </c>
+      <c r="E97">
+        <v>1</v>
+      </c>
+      <c r="F97" t="str">
+        <v>active</v>
+      </c>
+      <c r="G97" t="str">
+        <v>leadership_approach_q24::D::vision</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G65"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G97"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>